<commit_message>
fix(productos): el RD 1420/2006 (anisakis) está DEROGADO por el RD 1021/2022 (art. 8.1; cartel art. 8.2) — cita corregida en guía gastronómica (checklist-appcc C27/H27), pack APPCC (12: I13/B32 · 18: A46/A49/B28), 3 motores con gate anti-cita-derogada, 3 SPEC y 26 ficheros de la capa de producto (sushi-bar decía «RD 1420/2006 vigente»); kit-tareas sin cambios de celda
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kK9BRAxpAsfsxudgwH42U
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/guia-restaurante-gastronomico/budget-bodega.xlsx
+++ b/astro-site/public/dl/guia-restaurante-gastronomico/budget-bodega.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.00&quot;×&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +70,10 @@
       <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
+    </font>
+    <font/>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -123,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,6 +200,23 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -697,7 +718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T59"/>
+  <dimension ref="A1:T67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3440,123 +3461,327 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="24" t="inlineStr">
+      <c r="A55" s="32" t="inlineStr">
         <is>
           <t>RESUMEN Y PARÁMETROS — lo calcula el libro (v2.0)</t>
         </is>
       </c>
-      <c r="E55" s="22" t="n"/>
-      <c r="F55" s="22" t="n"/>
-      <c r="G55" s="22" t="n"/>
-      <c r="I55" s="25" t="n"/>
-      <c r="K55" s="25" t="n"/>
-      <c r="L55" s="21" t="n"/>
-      <c r="M55" s="21" t="n"/>
-      <c r="N55" s="22" t="n"/>
-      <c r="O55" s="22" t="n"/>
-      <c r="T55" s="22" t="n"/>
+      <c r="B55" s="33" t="n"/>
+      <c r="C55" s="33" t="n"/>
+      <c r="D55" s="33" t="n"/>
+      <c r="E55" s="34" t="n"/>
+      <c r="F55" s="34" t="n"/>
+      <c r="G55" s="34" t="n"/>
+      <c r="H55" s="33" t="n"/>
+      <c r="I55" s="35" t="n"/>
+      <c r="J55" s="33" t="n"/>
+      <c r="K55" s="35" t="n"/>
+      <c r="L55" s="36" t="n"/>
+      <c r="M55" s="36" t="n"/>
+      <c r="N55" s="34" t="n"/>
+      <c r="O55" s="34" t="n"/>
+      <c r="P55" s="33" t="n"/>
+      <c r="Q55" s="33" t="n"/>
+      <c r="R55" s="33" t="n"/>
+      <c r="S55" s="33" t="n"/>
+      <c r="T55" s="34" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="24" t="inlineStr">
+      <c r="A56" s="33" t="n"/>
+      <c r="B56" s="32" t="inlineStr">
         <is>
           <t>TOTAL BODEGA</t>
         </is>
       </c>
-      <c r="E56" s="22" t="n"/>
-      <c r="F56" s="22" t="n"/>
-      <c r="G56" s="22" t="n"/>
-      <c r="I56" s="26">
+      <c r="C56" s="33" t="n"/>
+      <c r="D56" s="33" t="n"/>
+      <c r="E56" s="34" t="n"/>
+      <c r="F56" s="34" t="n"/>
+      <c r="G56" s="34" t="n"/>
+      <c r="H56" s="33" t="n"/>
+      <c r="I56" s="37">
         <f>IF(COUNT(I5:I54)=0,"",SUM(I5:I54))</f>
         <v>306.0</v>
       </c>
-      <c r="K56" s="25" t="n"/>
-      <c r="L56" s="27">
+      <c r="J56" s="33" t="n"/>
+      <c r="K56" s="35" t="n"/>
+      <c r="L56" s="38">
         <f>IFERROR(IF(OR($O$56="",$O$56=0,$N$56=""),"",($O$56-$N$56)/$O$56),"")</f>
         <v>0.6382059800664452</v>
       </c>
-      <c r="M56" s="27">
+      <c r="M56" s="38">
         <f>IFERROR(IF(OR($N$56="",$O$56="",$O$56=0),"",$N$56/$O$56),"")</f>
         <v>0.36179401993355476</v>
       </c>
-      <c r="N56" s="28">
+      <c r="N56" s="39">
         <f>IF(COUNT(N5:N54)=0,"",SUM(N5:N54))</f>
         <v>3780.0</v>
       </c>
-      <c r="O56" s="28">
+      <c r="O56" s="39">
         <f>IF(COUNT(O5:O54)=0,"",SUM(O5:O54))</f>
         <v>10447.933884297523</v>
       </c>
-      <c r="T56" s="22" t="n"/>
+      <c r="P56" s="33" t="n"/>
+      <c r="Q56" s="33" t="n"/>
+      <c r="R56" s="33" t="n"/>
+      <c r="S56" s="33" t="n"/>
+      <c r="T56" s="34" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="29" t="inlineStr">
+      <c r="A57" s="40" t="inlineStr">
         <is>
           <t>El «Valor stock a coste» de la fila TOTAL es la cifra que alimenta la partida «Bodega inicial (vinos)» de plan-financiero-3-anos.xlsx, hoja «Inversión». Cópiala a mano: los libros no se enlazan entre sí porque un .xlsx movido de carpeta daría #REF! [TEC-19 · §4.3 · §1.13].</t>
         </is>
       </c>
-      <c r="B57" s="22" t="n"/>
-      <c r="C57" s="22" t="n"/>
-      <c r="D57" s="22" t="n"/>
-      <c r="E57" s="22" t="n"/>
-      <c r="F57" s="22" t="n"/>
-      <c r="G57" s="22" t="n"/>
-      <c r="H57" s="22" t="n"/>
-      <c r="I57" s="25" t="n"/>
-      <c r="J57" s="22" t="n"/>
-      <c r="K57" s="25" t="n"/>
-      <c r="L57" s="21" t="n"/>
-      <c r="M57" s="21" t="n"/>
-      <c r="N57" s="22" t="n"/>
-      <c r="O57" s="22" t="n"/>
-      <c r="P57" s="22" t="n"/>
-      <c r="Q57" s="22" t="n"/>
-      <c r="R57" s="22" t="n"/>
-      <c r="S57" s="22" t="n"/>
-      <c r="T57" s="22" t="n"/>
+      <c r="B57" s="34" t="n"/>
+      <c r="C57" s="34" t="n"/>
+      <c r="D57" s="34" t="n"/>
+      <c r="E57" s="34" t="n"/>
+      <c r="F57" s="34" t="n"/>
+      <c r="G57" s="34" t="n"/>
+      <c r="H57" s="34" t="n"/>
+      <c r="I57" s="35" t="n"/>
+      <c r="J57" s="34" t="n"/>
+      <c r="K57" s="35" t="n"/>
+      <c r="L57" s="36" t="n"/>
+      <c r="M57" s="36" t="n"/>
+      <c r="N57" s="34" t="n"/>
+      <c r="O57" s="34" t="n"/>
+      <c r="P57" s="34" t="n"/>
+      <c r="Q57" s="34" t="n"/>
+      <c r="R57" s="34" t="n"/>
+      <c r="S57" s="34" t="n"/>
+      <c r="T57" s="34" t="n"/>
     </row>
     <row r="58">
-      <c r="E58" s="22" t="n"/>
-      <c r="F58" s="22" t="n"/>
-      <c r="G58" s="22" t="n"/>
-      <c r="I58" s="25" t="n"/>
-      <c r="K58" s="25" t="n"/>
-      <c r="L58" s="21" t="n"/>
-      <c r="M58" s="21" t="n"/>
-      <c r="N58" s="22" t="n"/>
-      <c r="O58" s="22" t="n"/>
-      <c r="T58" s="22" t="n"/>
+      <c r="A58" s="33" t="n"/>
+      <c r="B58" s="33" t="n"/>
+      <c r="C58" s="33" t="n"/>
+      <c r="D58" s="33" t="n"/>
+      <c r="E58" s="34" t="n"/>
+      <c r="F58" s="34" t="n"/>
+      <c r="G58" s="34" t="n"/>
+      <c r="H58" s="33" t="n"/>
+      <c r="I58" s="35" t="n"/>
+      <c r="J58" s="33" t="n"/>
+      <c r="K58" s="35" t="n"/>
+      <c r="L58" s="36" t="n"/>
+      <c r="M58" s="36" t="n"/>
+      <c r="N58" s="34" t="n"/>
+      <c r="O58" s="34" t="n"/>
+      <c r="P58" s="33" t="n"/>
+      <c r="Q58" s="33" t="n"/>
+      <c r="R58" s="33" t="n"/>
+      <c r="S58" s="33" t="n"/>
+      <c r="T58" s="34" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="33" t="inlineStr">
         <is>
           <t>IVA de la bebida alcohólica (%)</t>
         </is>
       </c>
-      <c r="B59" s="21" t="n"/>
-      <c r="C59" s="30" t="n">
+      <c r="B59" s="36" t="n"/>
+      <c r="C59" s="41" t="n">
         <v>0.21</v>
       </c>
-      <c r="D59" s="31" t="inlineStr">
+      <c r="D59" s="42" t="inlineStr">
         <is>
           <t>21 % en bebidas alcohólicas (art. 91 de la Ley del IVA). El PVP de la columna F es el de CARTA, que en España se anuncia CON IVA: el multiplicador, el margen, el food cost y el valor a PVP se calculan sobre la columna «PVP sin IVA», no sobre el precio de carta.</t>
         </is>
       </c>
-      <c r="E59" s="22" t="n"/>
-      <c r="F59" s="22" t="n"/>
-      <c r="G59" s="22" t="n"/>
-      <c r="H59" s="21" t="n"/>
-      <c r="I59" s="25" t="n"/>
-      <c r="J59" s="21" t="n"/>
-      <c r="K59" s="25" t="n"/>
-      <c r="L59" s="21" t="n"/>
-      <c r="M59" s="21" t="n"/>
-      <c r="N59" s="22" t="n"/>
-      <c r="O59" s="22" t="n"/>
-      <c r="P59" s="21" t="n"/>
-      <c r="Q59" s="21" t="n"/>
-      <c r="R59" s="21" t="n"/>
-      <c r="S59" s="21" t="n"/>
-      <c r="T59" s="22" t="n"/>
+      <c r="E59" s="34" t="n"/>
+      <c r="F59" s="34" t="n"/>
+      <c r="G59" s="34" t="n"/>
+      <c r="H59" s="36" t="n"/>
+      <c r="I59" s="35" t="n"/>
+      <c r="J59" s="36" t="n"/>
+      <c r="K59" s="35" t="n"/>
+      <c r="L59" s="36" t="n"/>
+      <c r="M59" s="36" t="n"/>
+      <c r="N59" s="34" t="n"/>
+      <c r="O59" s="34" t="n"/>
+      <c r="P59" s="36" t="n"/>
+      <c r="Q59" s="36" t="n"/>
+      <c r="R59" s="36" t="n"/>
+      <c r="S59" s="36" t="n"/>
+      <c r="T59" s="34" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="33" t="n"/>
+      <c r="B60" s="33" t="n"/>
+      <c r="C60" s="33" t="n"/>
+      <c r="D60" s="33" t="n"/>
+      <c r="E60" s="34" t="n"/>
+      <c r="F60" s="34" t="n"/>
+      <c r="G60" s="34" t="n"/>
+      <c r="H60" s="33" t="n"/>
+      <c r="I60" s="35" t="n"/>
+      <c r="J60" s="33" t="n"/>
+      <c r="K60" s="35" t="n"/>
+      <c r="L60" s="36" t="n"/>
+      <c r="M60" s="36" t="n"/>
+      <c r="N60" s="34" t="n"/>
+      <c r="O60" s="34" t="n"/>
+      <c r="P60" s="33" t="n"/>
+      <c r="Q60" s="33" t="n"/>
+      <c r="R60" s="33" t="n"/>
+      <c r="S60" s="33" t="n"/>
+      <c r="T60" s="34" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="33" t="n"/>
+      <c r="B61" s="33" t="n"/>
+      <c r="C61" s="33" t="n"/>
+      <c r="D61" s="33" t="n"/>
+      <c r="E61" s="34" t="n"/>
+      <c r="F61" s="34" t="n"/>
+      <c r="G61" s="34" t="n"/>
+      <c r="H61" s="33" t="n"/>
+      <c r="I61" s="35" t="n"/>
+      <c r="J61" s="33" t="n"/>
+      <c r="K61" s="35" t="n"/>
+      <c r="L61" s="36" t="n"/>
+      <c r="M61" s="36" t="n"/>
+      <c r="N61" s="34" t="n"/>
+      <c r="O61" s="34" t="n"/>
+      <c r="P61" s="33" t="n"/>
+      <c r="Q61" s="33" t="n"/>
+      <c r="R61" s="33" t="n"/>
+      <c r="S61" s="33" t="n"/>
+      <c r="T61" s="34" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="33" t="n"/>
+      <c r="B62" s="33" t="n"/>
+      <c r="C62" s="33" t="n"/>
+      <c r="D62" s="33" t="n"/>
+      <c r="E62" s="34" t="n"/>
+      <c r="F62" s="34" t="n"/>
+      <c r="G62" s="34" t="n"/>
+      <c r="H62" s="33" t="n"/>
+      <c r="I62" s="35" t="n"/>
+      <c r="J62" s="33" t="n"/>
+      <c r="K62" s="35" t="n"/>
+      <c r="L62" s="36" t="n"/>
+      <c r="M62" s="36" t="n"/>
+      <c r="N62" s="34" t="n"/>
+      <c r="O62" s="34" t="n"/>
+      <c r="P62" s="33" t="n"/>
+      <c r="Q62" s="33" t="n"/>
+      <c r="R62" s="33" t="n"/>
+      <c r="S62" s="33" t="n"/>
+      <c r="T62" s="34" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="33" t="n"/>
+      <c r="B63" s="33" t="n"/>
+      <c r="C63" s="33" t="n"/>
+      <c r="D63" s="33" t="n"/>
+      <c r="E63" s="34" t="n"/>
+      <c r="F63" s="34" t="n"/>
+      <c r="G63" s="34" t="n"/>
+      <c r="H63" s="33" t="n"/>
+      <c r="I63" s="35" t="n"/>
+      <c r="J63" s="33" t="n"/>
+      <c r="K63" s="35" t="n"/>
+      <c r="L63" s="36" t="n"/>
+      <c r="M63" s="36" t="n"/>
+      <c r="N63" s="34" t="n"/>
+      <c r="O63" s="34" t="n"/>
+      <c r="P63" s="33" t="n"/>
+      <c r="Q63" s="33" t="n"/>
+      <c r="R63" s="33" t="n"/>
+      <c r="S63" s="33" t="n"/>
+      <c r="T63" s="34" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="33" t="n"/>
+      <c r="B64" s="33" t="n"/>
+      <c r="C64" s="33" t="n"/>
+      <c r="D64" s="33" t="n"/>
+      <c r="E64" s="34" t="n"/>
+      <c r="F64" s="34" t="n"/>
+      <c r="G64" s="34" t="n"/>
+      <c r="H64" s="33" t="n"/>
+      <c r="I64" s="35" t="n"/>
+      <c r="J64" s="33" t="n"/>
+      <c r="K64" s="35" t="n"/>
+      <c r="L64" s="36" t="n"/>
+      <c r="M64" s="36" t="n"/>
+      <c r="N64" s="34" t="n"/>
+      <c r="O64" s="34" t="n"/>
+      <c r="P64" s="33" t="n"/>
+      <c r="Q64" s="33" t="n"/>
+      <c r="R64" s="33" t="n"/>
+      <c r="S64" s="33" t="n"/>
+      <c r="T64" s="34" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="33" t="n"/>
+      <c r="B65" s="33" t="n"/>
+      <c r="C65" s="33" t="n"/>
+      <c r="D65" s="33" t="n"/>
+      <c r="E65" s="34" t="n"/>
+      <c r="F65" s="34" t="n"/>
+      <c r="G65" s="34" t="n"/>
+      <c r="H65" s="33" t="n"/>
+      <c r="I65" s="35" t="n"/>
+      <c r="J65" s="33" t="n"/>
+      <c r="K65" s="35" t="n"/>
+      <c r="L65" s="36" t="n"/>
+      <c r="M65" s="36" t="n"/>
+      <c r="N65" s="34" t="n"/>
+      <c r="O65" s="34" t="n"/>
+      <c r="P65" s="33" t="n"/>
+      <c r="Q65" s="33" t="n"/>
+      <c r="R65" s="33" t="n"/>
+      <c r="S65" s="33" t="n"/>
+      <c r="T65" s="34" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="33" t="n"/>
+      <c r="B66" s="33" t="n"/>
+      <c r="C66" s="33" t="n"/>
+      <c r="D66" s="33" t="n"/>
+      <c r="E66" s="34" t="n"/>
+      <c r="F66" s="34" t="n"/>
+      <c r="G66" s="34" t="n"/>
+      <c r="H66" s="33" t="n"/>
+      <c r="I66" s="35" t="n"/>
+      <c r="J66" s="33" t="n"/>
+      <c r="K66" s="35" t="n"/>
+      <c r="L66" s="36" t="n"/>
+      <c r="M66" s="36" t="n"/>
+      <c r="N66" s="34" t="n"/>
+      <c r="O66" s="34" t="n"/>
+      <c r="P66" s="33" t="n"/>
+      <c r="Q66" s="33" t="n"/>
+      <c r="R66" s="33" t="n"/>
+      <c r="S66" s="33" t="n"/>
+      <c r="T66" s="34" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="33" t="n"/>
+      <c r="B67" s="33" t="n"/>
+      <c r="C67" s="33" t="n"/>
+      <c r="D67" s="33" t="n"/>
+      <c r="E67" s="34" t="n"/>
+      <c r="F67" s="34" t="n"/>
+      <c r="G67" s="34" t="n"/>
+      <c r="H67" s="33" t="n"/>
+      <c r="I67" s="35" t="n"/>
+      <c r="J67" s="33" t="n"/>
+      <c r="K67" s="35" t="n"/>
+      <c r="L67" s="36" t="n"/>
+      <c r="M67" s="36" t="n"/>
+      <c r="N67" s="34" t="n"/>
+      <c r="O67" s="34" t="n"/>
+      <c r="P67" s="33" t="n"/>
+      <c r="Q67" s="33" t="n"/>
+      <c r="R67" s="33" t="n"/>
+      <c r="S67" s="33" t="n"/>
+      <c r="T67" s="34" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>

</xml_diff>